<commit_message>
Updated Excel template for deprecation report
</commit_message>
<xml_diff>
--- a/jeaf-generator/src/main/resources/Deprecation_Report_Template.xlsx
+++ b/jeaf-generator/src/main/resources/Deprecation_Report_Template.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10531"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10821"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tillmann.schall/Projects/JEAF/jeaf-generator/jeaf-generator/src/main/resources/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2EC330ED-BB34-4043-A273-9B77F23749F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{940AF31E-6AD2-F249-98B2-260B852C4C26}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="36860" yWindow="2360" windowWidth="51160" windowHeight="28140" xr2:uid="{441949ED-3404-8548-92CD-A40A7EA6D1DC}"/>
+    <workbookView xWindow="36860" yWindow="660" windowWidth="51160" windowHeight="28140" xr2:uid="{441949ED-3404-8548-92CD-A40A7EA6D1DC}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -41,9 +41,6 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
   <si>
-    <t>Type</t>
-  </si>
-  <si>
     <t>Package</t>
   </si>
   <si>
@@ -63,6 +60,9 @@
   </si>
   <si>
     <t>Removal Date</t>
+  </si>
+  <si>
+    <t>Element</t>
   </si>
 </sst>
 </file>
@@ -145,25 +145,25 @@
     <xf numFmtId="164" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
@@ -181,12 +181,6 @@
     </dxf>
     <dxf>
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="top" textRotation="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="top" textRotation="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <alignment vertical="top" textRotation="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -216,11 +210,17 @@
       </border>
     </dxf>
     <dxf>
+      <alignment vertical="top" textRotation="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
       <border outline="0">
         <bottom style="thin">
           <color theme="4"/>
         </bottom>
       </border>
+    </dxf>
+    <dxf>
+      <alignment vertical="top" textRotation="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -236,13 +236,13 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{5FC88E85-2BB1-CD48-A0D0-BB78642BF973}" name="Table1" displayName="Table1" ref="A1:H1048576" totalsRowShown="0" headerRowDxfId="5" dataDxfId="4" headerRowBorderDxfId="11" tableBorderDxfId="10">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{5FC88E85-2BB1-CD48-A0D0-BB78642BF973}" name="Table1" displayName="Table1" ref="A1:H1048576" totalsRowShown="0" headerRowDxfId="11" dataDxfId="9" headerRowBorderDxfId="10" tableBorderDxfId="8">
   <autoFilter ref="A1:H1048576" xr:uid="{5FC88E85-2BB1-CD48-A0D0-BB78642BF973}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{A4DDCCBB-E133-DF45-8389-C4AD19D8AEB7}" name="Type" dataDxfId="9"/>
-    <tableColumn id="2" xr3:uid="{439690A4-77A7-D848-A33C-19AF8EF0CF49}" name="Package" dataDxfId="8"/>
-    <tableColumn id="3" xr3:uid="{BC971382-1AD8-4C4D-972D-DF92F8F0260A}" name="Property / Operation" dataDxfId="7"/>
-    <tableColumn id="4" xr3:uid="{5A67E0BD-2295-9F48-B6C2-59EBC6AF29B1}" name="HTTP Header" dataDxfId="6"/>
+    <tableColumn id="1" xr3:uid="{A4DDCCBB-E133-DF45-8389-C4AD19D8AEB7}" name="Element" dataDxfId="7"/>
+    <tableColumn id="2" xr3:uid="{439690A4-77A7-D848-A33C-19AF8EF0CF49}" name="Package" dataDxfId="6"/>
+    <tableColumn id="3" xr3:uid="{BC971382-1AD8-4C4D-972D-DF92F8F0260A}" name="Property / Operation" dataDxfId="5"/>
+    <tableColumn id="4" xr3:uid="{5A67E0BD-2295-9F48-B6C2-59EBC6AF29B1}" name="HTTP Header" dataDxfId="4"/>
     <tableColumn id="5" xr3:uid="{1DDDD3D3-BC66-DB4E-A899-65EA0DA59605}" name="Description" dataDxfId="3"/>
     <tableColumn id="6" xr3:uid="{122F67FD-2569-C44A-A432-EAFF5935108B}" name="Deprecated since" dataDxfId="2"/>
     <tableColumn id="7" xr3:uid="{4B86B03A-67C7-E347-8943-3AB848258236}" name="Planned to be removed" dataDxfId="1"/>
@@ -582,28 +582,28 @@
   <sheetData>
     <row r="1" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="F1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="G1" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="H1" s="4" t="s">
         <v>6</v>
-      </c>
-      <c r="H1" s="4" t="s">
-        <v>7</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">

</xml_diff>